<commit_message>
Add resale prices to Phase 3 parts from RFQ 1139539
- 40 Phase 3 parts updated with resale prices
- Enables margin analysis in sourcing output

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -2051,6 +2051,9 @@
       <c r="F50">
         <v>33.25</v>
       </c>
+      <c r="G50">
+        <v>33.25</v>
+      </c>
       <c r="H50">
         <v>0</v>
       </c>
@@ -11284,7 +11287,7 @@
         <v>34.8</v>
       </c>
       <c r="G328">
-        <v>42.4390243902439</v>
+        <v>34.8</v>
       </c>
       <c r="H328">
         <v>50</v>
@@ -21162,6 +21165,9 @@
       <c r="F619">
         <v>7.45</v>
       </c>
+      <c r="G619">
+        <v>7.45</v>
+      </c>
       <c r="H619">
         <v>0</v>
       </c>
@@ -21208,6 +21214,9 @@
       <c r="F621">
         <v>13.5</v>
       </c>
+      <c r="G621">
+        <v>13.5</v>
+      </c>
       <c r="H621">
         <v>0</v>
       </c>
@@ -21254,6 +21263,9 @@
       <c r="F623">
         <v>9.36</v>
       </c>
+      <c r="G623">
+        <v>9.36</v>
+      </c>
       <c r="H623">
         <v>0</v>
       </c>
@@ -21315,6 +21327,9 @@
       <c r="F625">
         <v>7.66</v>
       </c>
+      <c r="G625">
+        <v>7.66</v>
+      </c>
       <c r="H625">
         <v>0</v>
       </c>
@@ -21341,6 +21356,9 @@
       <c r="F626">
         <v>22.77</v>
       </c>
+      <c r="G626">
+        <v>22.77</v>
+      </c>
       <c r="H626">
         <v>0</v>
       </c>
@@ -22597,7 +22615,7 @@
         <v>5.62</v>
       </c>
       <c r="G664">
-        <v>6.853658536585367</v>
+        <v>5.62</v>
       </c>
       <c r="H664">
         <v>300</v>
@@ -40485,6 +40503,9 @@
       <c r="F1192">
         <v>109.27</v>
       </c>
+      <c r="G1192">
+        <v>109.27</v>
+      </c>
       <c r="H1192">
         <v>0</v>
       </c>
@@ -40954,7 +40975,7 @@
         <v>2.72</v>
       </c>
       <c r="G1207">
-        <v>3.4692</v>
+        <v>2.72</v>
       </c>
       <c r="H1207">
         <v>140</v>
@@ -42140,6 +42161,9 @@
       <c r="F1244">
         <v>23.54</v>
       </c>
+      <c r="G1244">
+        <v>23.54</v>
+      </c>
       <c r="H1244">
         <v>20</v>
       </c>
@@ -42211,7 +42235,7 @@
         <v>6.81</v>
       </c>
       <c r="G1246">
-        <v>0</v>
+        <v>6.81</v>
       </c>
       <c r="H1246">
         <v>1</v>
@@ -42261,7 +42285,7 @@
         <v>1.78</v>
       </c>
       <c r="G1247">
-        <v>0</v>
+        <v>1.78</v>
       </c>
       <c r="H1247">
         <v>1</v>
@@ -42311,7 +42335,7 @@
         <v>21.17</v>
       </c>
       <c r="G1248">
-        <v>0</v>
+        <v>21.17</v>
       </c>
       <c r="H1248">
         <v>1</v>
@@ -42361,7 +42385,7 @@
         <v>0.26</v>
       </c>
       <c r="G1249">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="H1249">
         <v>1</v>
@@ -42411,7 +42435,7 @@
         <v>0.31</v>
       </c>
       <c r="G1250">
-        <v>0</v>
+        <v>0.31</v>
       </c>
       <c r="H1250">
         <v>1</v>
@@ -42461,7 +42485,7 @@
         <v>87.64</v>
       </c>
       <c r="G1251">
-        <v>0</v>
+        <v>87.64</v>
       </c>
       <c r="H1251">
         <v>1</v>
@@ -42511,7 +42535,7 @@
         <v>9.8</v>
       </c>
       <c r="G1252">
-        <v>0</v>
+        <v>9.8</v>
       </c>
       <c r="H1252">
         <v>1</v>
@@ -42561,7 +42585,7 @@
         <v>0.05</v>
       </c>
       <c r="G1253">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H1253">
         <v>1</v>
@@ -42611,7 +42635,7 @@
         <v>18.96</v>
       </c>
       <c r="G1254">
-        <v>0</v>
+        <v>18.96</v>
       </c>
       <c r="H1254">
         <v>1</v>
@@ -42661,7 +42685,7 @@
         <v>7.38</v>
       </c>
       <c r="G1255">
-        <v>0</v>
+        <v>7.38</v>
       </c>
       <c r="H1255">
         <v>1</v>
@@ -42711,7 +42735,7 @@
         <v>4.7</v>
       </c>
       <c r="G1256">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="H1256">
         <v>1</v>
@@ -42761,7 +42785,7 @@
         <v>5.69</v>
       </c>
       <c r="G1257">
-        <v>0</v>
+        <v>5.69</v>
       </c>
       <c r="H1257">
         <v>1</v>
@@ -42811,7 +42835,7 @@
         <v>2.4</v>
       </c>
       <c r="G1258">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="H1258">
         <v>1</v>
@@ -42861,7 +42885,7 @@
         <v>3.35</v>
       </c>
       <c r="G1259">
-        <v>0</v>
+        <v>3.35</v>
       </c>
       <c r="H1259">
         <v>1</v>
@@ -42911,7 +42935,7 @@
         <v>0.45</v>
       </c>
       <c r="G1260">
-        <v>0</v>
+        <v>5.34</v>
       </c>
       <c r="H1260">
         <v>1</v>
@@ -42961,7 +42985,7 @@
         <v>5.34</v>
       </c>
       <c r="G1261">
-        <v>0</v>
+        <v>2.61</v>
       </c>
       <c r="H1261">
         <v>1</v>
@@ -43011,7 +43035,7 @@
         <v>2.61</v>
       </c>
       <c r="G1262">
-        <v>0</v>
+        <v>1.49</v>
       </c>
       <c r="H1262">
         <v>1</v>
@@ -43061,7 +43085,7 @@
         <v>1.49</v>
       </c>
       <c r="G1263">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="H1263">
         <v>1</v>
@@ -43111,7 +43135,7 @@
         <v>0.39</v>
       </c>
       <c r="G1264">
-        <v>0</v>
+        <v>1.59</v>
       </c>
       <c r="H1264">
         <v>1</v>
@@ -43161,7 +43185,7 @@
         <v>1.59</v>
       </c>
       <c r="G1265">
-        <v>0</v>
+        <v>6.98</v>
       </c>
       <c r="H1265">
         <v>1</v>
@@ -43211,7 +43235,7 @@
         <v>6.98</v>
       </c>
       <c r="G1266">
-        <v>0</v>
+        <v>31.31</v>
       </c>
       <c r="H1266">
         <v>1</v>
@@ -43261,7 +43285,7 @@
         <v>31.31</v>
       </c>
       <c r="G1267">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="H1267">
         <v>1</v>
@@ -43311,7 +43335,7 @@
         <v>0.11</v>
       </c>
       <c r="G1268">
-        <v>0</v>
+        <v>9.8</v>
       </c>
       <c r="H1268">
         <v>1</v>
@@ -43361,7 +43385,7 @@
         <v>9.8</v>
       </c>
       <c r="G1269">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="H1269">
         <v>1</v>
@@ -43411,7 +43435,7 @@
         <v>0.63</v>
       </c>
       <c r="G1270">
-        <v>0</v>
+        <v>0.89</v>
       </c>
       <c r="H1270">
         <v>1</v>
@@ -43461,7 +43485,7 @@
         <v>0.89</v>
       </c>
       <c r="G1271">
-        <v>0</v>
+        <v>1.29</v>
       </c>
       <c r="H1271">
         <v>1</v>
@@ -43511,7 +43535,7 @@
         <v>1.29</v>
       </c>
       <c r="G1272">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="H1272">
         <v>1</v>
@@ -43561,7 +43585,7 @@
         <v>0.15</v>
       </c>
       <c r="G1273">
-        <v>0</v>
+        <v>9.32</v>
       </c>
       <c r="H1273">
         <v>1</v>
@@ -43611,7 +43635,7 @@
         <v>9.32</v>
       </c>
       <c r="G1274">
-        <v>0</v>
+        <v>12.64</v>
       </c>
       <c r="H1274">
         <v>1</v>
@@ -43661,7 +43685,7 @@
         <v>12.64</v>
       </c>
       <c r="G1275">
-        <v>0</v>
+        <v>2.85</v>
       </c>
       <c r="H1275">
         <v>1</v>
@@ -43711,7 +43735,7 @@
         <v>2.85</v>
       </c>
       <c r="G1276">
-        <v>0</v>
+        <v>10.24</v>
       </c>
       <c r="H1276">
         <v>1</v>
@@ -43761,7 +43785,7 @@
         <v>10.24</v>
       </c>
       <c r="G1277">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="H1277">
         <v>1</v>

</xml_diff>

<commit_message>
Update Phase 3 MOQs from RFQ 1139539
- 40 Phase 3 parts updated with correct MOQs
- Also sets Reorder Threshold = MOQ where not already set

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -2055,7 +2055,10 @@
         <v>33.25</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="J50">
+        <v>100</v>
       </c>
       <c r="L50" t="str">
         <v>New Award</v>
@@ -11295,6 +11298,9 @@
       <c r="I328" t="str">
         <v>10 weeks</v>
       </c>
+      <c r="J328">
+        <v>50</v>
+      </c>
       <c r="L328" t="str">
         <v>New Award</v>
       </c>
@@ -21169,7 +21175,10 @@
         <v>7.45</v>
       </c>
       <c r="H619">
-        <v>0</v>
+        <v>500</v>
+      </c>
+      <c r="J619">
+        <v>500</v>
       </c>
       <c r="L619" t="str">
         <v>New Award</v>
@@ -21218,7 +21227,10 @@
         <v>13.5</v>
       </c>
       <c r="H621">
-        <v>0</v>
+        <v>250</v>
+      </c>
+      <c r="J621">
+        <v>250</v>
       </c>
       <c r="L621" t="str">
         <v>New Award</v>
@@ -21267,7 +21279,10 @@
         <v>9.36</v>
       </c>
       <c r="H623">
-        <v>0</v>
+        <v>250</v>
+      </c>
+      <c r="J623">
+        <v>250</v>
       </c>
       <c r="L623" t="str">
         <v>New Award</v>
@@ -21331,7 +21346,10 @@
         <v>7.66</v>
       </c>
       <c r="H625">
-        <v>0</v>
+        <v>250</v>
+      </c>
+      <c r="J625">
+        <v>250</v>
       </c>
       <c r="L625" t="str">
         <v>New Award</v>
@@ -21360,7 +21378,10 @@
         <v>22.77</v>
       </c>
       <c r="H626">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="J626">
+        <v>50</v>
       </c>
       <c r="L626" t="str">
         <v>New Award</v>
@@ -22618,10 +22639,13 @@
         <v>5.62</v>
       </c>
       <c r="H664">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="I664" t="str">
         <v>5 weeks</v>
+      </c>
+      <c r="J664">
+        <v>500</v>
       </c>
       <c r="L664" t="str">
         <v>New Award</v>
@@ -40507,7 +40531,10 @@
         <v>109.27</v>
       </c>
       <c r="H1192">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="J1192">
+        <v>10</v>
       </c>
       <c r="L1192" t="str">
         <v>New Award</v>
@@ -42238,13 +42265,13 @@
         <v>6.81</v>
       </c>
       <c r="H1246">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1246" t="str">
         <v/>
       </c>
       <c r="J1246">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1246" t="str">
         <v>Jake Harris</v>
@@ -42288,13 +42315,13 @@
         <v>1.78</v>
       </c>
       <c r="H1247">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="I1247" t="str">
         <v/>
       </c>
       <c r="J1247">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="K1247" t="str">
         <v>Jake Harris</v>
@@ -42338,13 +42365,13 @@
         <v>21.17</v>
       </c>
       <c r="H1248">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="I1248" t="str">
         <v/>
       </c>
       <c r="J1248">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K1248" t="str">
         <v>Jake Harris</v>
@@ -42388,13 +42415,13 @@
         <v>0.26</v>
       </c>
       <c r="H1249">
-        <v>1</v>
+        <v>1500</v>
       </c>
       <c r="I1249" t="str">
         <v/>
       </c>
       <c r="J1249">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="K1249" t="str">
         <v>Jake Harris</v>
@@ -42438,13 +42465,13 @@
         <v>0.31</v>
       </c>
       <c r="H1250">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1250" t="str">
         <v/>
       </c>
       <c r="J1250">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K1250" t="str">
         <v>Jake Harris</v>
@@ -42488,13 +42515,13 @@
         <v>87.64</v>
       </c>
       <c r="H1251">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I1251" t="str">
         <v/>
       </c>
       <c r="J1251">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K1251" t="str">
         <v>Jake Harris</v>
@@ -42538,13 +42565,13 @@
         <v>9.8</v>
       </c>
       <c r="H1252">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="I1252" t="str">
         <v/>
       </c>
       <c r="J1252">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K1252" t="str">
         <v>Jake Harris</v>
@@ -42588,13 +42615,13 @@
         <v>0.05</v>
       </c>
       <c r="H1253">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="I1253" t="str">
         <v/>
       </c>
       <c r="J1253">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K1253" t="str">
         <v>Jake Harris</v>
@@ -42638,13 +42665,13 @@
         <v>18.96</v>
       </c>
       <c r="H1254">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="I1254" t="str">
         <v/>
       </c>
       <c r="J1254">
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="K1254" t="str">
         <v>Jake Harris</v>
@@ -42688,13 +42715,13 @@
         <v>7.38</v>
       </c>
       <c r="H1255">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="I1255" t="str">
         <v/>
       </c>
       <c r="J1255">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="K1255" t="str">
         <v>Jake Harris</v>
@@ -42738,13 +42765,13 @@
         <v>4.7</v>
       </c>
       <c r="H1256">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1256" t="str">
         <v/>
       </c>
       <c r="J1256">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1256" t="str">
         <v>Jake Harris</v>
@@ -42788,13 +42815,13 @@
         <v>5.69</v>
       </c>
       <c r="H1257">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="I1257" t="str">
         <v/>
       </c>
       <c r="J1257">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="K1257" t="str">
         <v>Jake Harris</v>
@@ -42838,13 +42865,13 @@
         <v>2.4</v>
       </c>
       <c r="H1258">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="I1258" t="str">
         <v/>
       </c>
       <c r="J1258">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="K1258" t="str">
         <v>Jake Harris</v>
@@ -42888,13 +42915,13 @@
         <v>3.35</v>
       </c>
       <c r="H1259">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1259" t="str">
         <v/>
       </c>
       <c r="J1259">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K1259" t="str">
         <v>Jake Harris</v>
@@ -42938,13 +42965,13 @@
         <v>5.34</v>
       </c>
       <c r="H1260">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1260" t="str">
         <v/>
       </c>
       <c r="J1260">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K1260" t="str">
         <v>Jake Harris</v>
@@ -42988,13 +43015,13 @@
         <v>2.61</v>
       </c>
       <c r="H1261">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1261" t="str">
         <v/>
       </c>
       <c r="J1261">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K1261" t="str">
         <v>Jake Harris</v>
@@ -43038,13 +43065,13 @@
         <v>1.49</v>
       </c>
       <c r="H1262">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="I1262" t="str">
         <v/>
       </c>
       <c r="J1262">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K1262" t="str">
         <v>Jake Harris</v>
@@ -43088,13 +43115,13 @@
         <v>0.39</v>
       </c>
       <c r="H1263">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1263" t="str">
         <v/>
       </c>
       <c r="J1263">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K1263" t="str">
         <v>Jake Harris</v>
@@ -43138,13 +43165,13 @@
         <v>1.59</v>
       </c>
       <c r="H1264">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="I1264" t="str">
         <v/>
       </c>
       <c r="J1264">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K1264" t="str">
         <v>Jake Harris</v>
@@ -43188,13 +43215,13 @@
         <v>6.98</v>
       </c>
       <c r="H1265">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1265" t="str">
         <v/>
       </c>
       <c r="J1265">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1265" t="str">
         <v>Jake Harris</v>
@@ -43238,13 +43265,13 @@
         <v>31.31</v>
       </c>
       <c r="H1266">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="I1266" t="str">
         <v/>
       </c>
       <c r="J1266">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="K1266" t="str">
         <v>Jake Harris</v>
@@ -43288,13 +43315,13 @@
         <v>0.11</v>
       </c>
       <c r="H1267">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="I1267" t="str">
         <v/>
       </c>
       <c r="J1267">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="K1267" t="str">
         <v>Jake Harris</v>
@@ -43338,13 +43365,13 @@
         <v>9.8</v>
       </c>
       <c r="H1268">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I1268" t="str">
         <v/>
       </c>
       <c r="J1268">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K1268" t="str">
         <v>Jake Harris</v>
@@ -43388,13 +43415,13 @@
         <v>0.63</v>
       </c>
       <c r="H1269">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="I1269" t="str">
         <v/>
       </c>
       <c r="J1269">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="K1269" t="str">
         <v>Jake Harris</v>
@@ -43438,13 +43465,13 @@
         <v>0.89</v>
       </c>
       <c r="H1270">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1270" t="str">
         <v/>
       </c>
       <c r="J1270">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K1270" t="str">
         <v>Jake Harris</v>
@@ -43488,13 +43515,13 @@
         <v>1.29</v>
       </c>
       <c r="H1271">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="I1271" t="str">
         <v/>
       </c>
       <c r="J1271">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="K1271" t="str">
         <v>Jake Harris</v>
@@ -43538,13 +43565,13 @@
         <v>0.15</v>
       </c>
       <c r="H1272">
-        <v>1</v>
+        <v>4000</v>
       </c>
       <c r="I1272" t="str">
         <v/>
       </c>
       <c r="J1272">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="K1272" t="str">
         <v>Jake Harris</v>
@@ -43588,13 +43615,13 @@
         <v>9.32</v>
       </c>
       <c r="H1273">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1273" t="str">
         <v/>
       </c>
       <c r="J1273">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1273" t="str">
         <v>Jake Harris</v>
@@ -43638,13 +43665,13 @@
         <v>12.64</v>
       </c>
       <c r="H1274">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1274" t="str">
         <v/>
       </c>
       <c r="J1274">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1274" t="str">
         <v>Jake Harris</v>
@@ -43688,13 +43715,13 @@
         <v>2.85</v>
       </c>
       <c r="H1275">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1275" t="str">
         <v/>
       </c>
       <c r="J1275">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1275" t="str">
         <v>Jake Harris</v>
@@ -43738,13 +43765,13 @@
         <v>10.24</v>
       </c>
       <c r="H1276">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I1276" t="str">
         <v/>
       </c>
       <c r="J1276">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K1276" t="str">
         <v>Jake Harris</v>
@@ -43788,13 +43815,13 @@
         <v>3.1</v>
       </c>
       <c r="H1277">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1277" t="str">
         <v/>
       </c>
       <c r="J1277">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K1277" t="str">
         <v>Jake Harris</v>

</xml_diff>

<commit_message>
Fix Phase 3 roster data from RFQ 1139539
- Fixed 22 rows with wrong CPC-to-MPN mappings
- Added missing CPC 29-178970-00 (ECEA1VKS470)
- Added check-phase3-roster.js for validation

Root cause: Original file sent had scrambled CPC-MPN assignments.
Fix: Cross-referenced RFQ 1139539 to correct all mappings.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1277"/>
+  <dimension ref="A1:P1278"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22621,10 +22621,10 @@
         <v>668-096777-009</v>
       </c>
       <c r="B664" t="str">
-        <v>K85X-ED-9P-CBR</v>
+        <v>DLS 1XP4AA35X</v>
       </c>
       <c r="C664" t="str">
-        <v>KYCON, INC</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH</v>
       </c>
       <c r="D664" t="str">
         <v>CONN,DSUB,9P,M,STR,BRD LCK,ROHS</v>
@@ -42177,7 +42177,7 @@
         <v>ADS8509IDW</v>
       </c>
       <c r="C1244" t="str">
-        <v>TEXAS INSTRUMENTS</v>
+        <v>TEXAS INSTRUMENTS (P)</v>
       </c>
       <c r="D1244" t="str">
         <v>IC,SMD,16 BIT SERIAL ADC,ROHS</v>
@@ -42250,7 +42250,7 @@
         <v>PTS120601B100R</v>
       </c>
       <c r="C1246" t="str">
-        <v>Vishay</v>
+        <v>VISHAY (P)</v>
       </c>
       <c r="D1246" t="str">
         <v/>
@@ -42500,7 +42500,7 @@
         <v>3838C2R7AP722X</v>
       </c>
       <c r="C1251" t="str">
-        <v>Passive Plus</v>
+        <v>PASSIVE PLUS INC. (P)</v>
       </c>
       <c r="D1251" t="str">
         <v/>
@@ -42947,10 +42947,10 @@
         <v>630-272519-001</v>
       </c>
       <c r="B1260" t="str">
-        <v>ECEA1VKS470</v>
+        <v>OPA2192IDGKT</v>
       </c>
       <c r="C1260" t="str">
-        <v>Panasonic</v>
+        <v>TEXAS INSTRUMENTS (P)</v>
       </c>
       <c r="D1260" t="str">
         <v/>
@@ -42997,7 +42997,7 @@
         <v>630-341490-001</v>
       </c>
       <c r="B1261" t="str">
-        <v>OPA2192IDGKT</v>
+        <v>TPS26620DRCT</v>
       </c>
       <c r="C1261" t="str">
         <v>TEXAS INSTRUMENTS (P)</v>
@@ -43047,7 +43047,7 @@
         <v>630-265677-001</v>
       </c>
       <c r="B1262" t="str">
-        <v>TPS26620DRCT</v>
+        <v>LM2941SX/NOPB</v>
       </c>
       <c r="C1262" t="str">
         <v>TEXAS INSTRUMENTS (P)</v>
@@ -43097,10 +43097,10 @@
         <v>648-130628-001</v>
       </c>
       <c r="B1263" t="str">
-        <v>LM2941SX/NOPB</v>
+        <v>EMVH500ADA101MJA0G</v>
       </c>
       <c r="C1263" t="str">
-        <v>TEXAS INSTRUMENTS (P)</v>
+        <v>NIPPON CHEMI-CON CORPORATION (A)</v>
       </c>
       <c r="D1263" t="str">
         <v/>
@@ -43147,10 +43147,10 @@
         <v>662-060106-012</v>
       </c>
       <c r="B1264" t="str">
-        <v>EMVH500ADA101MJA0G</v>
+        <v>555-2401F</v>
       </c>
       <c r="C1264" t="str">
-        <v>Nippon Chemi-Con Corporation</v>
+        <v>DIALIGHT (P)</v>
       </c>
       <c r="D1264" t="str">
         <v/>
@@ -43197,10 +43197,10 @@
         <v>630-096581-001</v>
       </c>
       <c r="B1265" t="str">
-        <v>555-2401F</v>
+        <v>LT1013DS8#PBF</v>
       </c>
       <c r="C1265" t="str">
-        <v>DIALIGHT (P)</v>
+        <v>ANALOG DEVICES INC. (P)</v>
       </c>
       <c r="D1265" t="str">
         <v/>
@@ -43247,10 +43247,10 @@
         <v>644-338613-001</v>
       </c>
       <c r="B1266" t="str">
-        <v>LT1013DS8#PBF</v>
+        <v>CX480D5</v>
       </c>
       <c r="C1266" t="str">
-        <v>ANALOG DEVICES INC. (P)</v>
+        <v>CRYDOM (P)</v>
       </c>
       <c r="D1266" t="str">
         <v/>
@@ -43297,10 +43297,10 @@
         <v>615-068556-200</v>
       </c>
       <c r="B1267" t="str">
-        <v>CX480D5</v>
+        <v>ERJ-3RQF2R0V</v>
       </c>
       <c r="C1267" t="str">
-        <v>CRYDOM (P)</v>
+        <v>PANASONIC (P)</v>
       </c>
       <c r="D1267" t="str">
         <v/>
@@ -43347,10 +43347,10 @@
         <v>668-132368-015</v>
       </c>
       <c r="B1268" t="str">
-        <v>ERJ-3RQF2R0V</v>
+        <v>164A16579X</v>
       </c>
       <c r="C1268" t="str">
-        <v>Panasonic</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH (P)</v>
       </c>
       <c r="D1268" t="str">
         <v/>
@@ -43397,10 +43397,10 @@
         <v>648-314833-001</v>
       </c>
       <c r="B1269" t="str">
-        <v>164A16579X</v>
+        <v>C3216X7R1V475K160AB</v>
       </c>
       <c r="C1269" t="str">
-        <v>CONEC Elektronische Bauelemente GmbH</v>
+        <v>TDK (P)</v>
       </c>
       <c r="D1269" t="str">
         <v/>
@@ -43447,10 +43447,10 @@
         <v>615-224835-010</v>
       </c>
       <c r="B1270" t="str">
-        <v>C3216X7R1V475K160AB</v>
+        <v>PATT0603E4991BGT1</v>
       </c>
       <c r="C1270" t="str">
-        <v>TDK (P)</v>
+        <v>VISHAY (P)</v>
       </c>
       <c r="D1270" t="str">
         <v/>
@@ -43497,10 +43497,10 @@
         <v>639-B70524-101</v>
       </c>
       <c r="B1271" t="str">
-        <v>PATT0603E4991BGT1</v>
+        <v>SRR1208-101KL</v>
       </c>
       <c r="C1271" t="str">
-        <v>Vishay</v>
+        <v>BOURNS (P)</v>
       </c>
       <c r="D1271" t="str">
         <v/>
@@ -43547,10 +43547,10 @@
         <v>648-162696-004</v>
       </c>
       <c r="B1272" t="str">
-        <v>SRR1208-101KL</v>
+        <v>C1608X5R1V474K080AB</v>
       </c>
       <c r="C1272" t="str">
-        <v>BOURNS (P)</v>
+        <v>TDK (P)</v>
       </c>
       <c r="D1272" t="str">
         <v/>
@@ -43597,10 +43597,10 @@
         <v>671-084849-001</v>
       </c>
       <c r="B1273" t="str">
-        <v>C1608X5R1V474K080AB</v>
+        <v>40.1151</v>
       </c>
       <c r="C1273" t="str">
-        <v>TDK (P)</v>
+        <v>SCHURTER (P)</v>
       </c>
       <c r="D1273" t="str">
         <v/>
@@ -43647,10 +43647,10 @@
         <v>630-311553-001</v>
       </c>
       <c r="B1274" t="str">
-        <v>40.1151</v>
+        <v>DP83630SQ/NOPB</v>
       </c>
       <c r="C1274" t="str">
-        <v>SCHURTER (P)</v>
+        <v>TEXAS INSTRUMENTS (P)</v>
       </c>
       <c r="D1274" t="str">
         <v/>
@@ -43697,10 +43697,10 @@
         <v>630-212275-001</v>
       </c>
       <c r="B1275" t="str">
-        <v>DP83630SQ/NOPB</v>
+        <v>L6491</v>
       </c>
       <c r="C1275" t="str">
-        <v>TEXAS INSTRUMENTS (P)</v>
+        <v>STMICROELECTRONICS (P)</v>
       </c>
       <c r="D1275" t="str">
         <v/>
@@ -43747,10 +43747,10 @@
         <v>668-C03283-001</v>
       </c>
       <c r="B1276" t="str">
-        <v>L6491</v>
+        <v>302W2CPXX72E40X</v>
       </c>
       <c r="C1276" t="str">
-        <v>STMICROELECTRONICS (P)</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH</v>
       </c>
       <c r="D1276" t="str">
         <v/>
@@ -43797,10 +43797,10 @@
         <v>785-088248-001</v>
       </c>
       <c r="B1277" t="str">
-        <v>302W2CPXX72E40X</v>
+        <v>ORDER TO SPECIFICATION</v>
       </c>
       <c r="C1277" t="str">
-        <v>CONEC Elektronische Bauelemente GmbH</v>
+        <v>ORDER TO SPECIFICATION (P)</v>
       </c>
       <c r="D1277" t="str">
         <v/>
@@ -43842,9 +43842,59 @@
         <v>2026-07-17</v>
       </c>
     </row>
+    <row r="1278">
+      <c r="A1278" t="str">
+        <v>29-178970-00</v>
+      </c>
+      <c r="B1278" t="str">
+        <v>ECEA1VKS470</v>
+      </c>
+      <c r="C1278" t="str">
+        <v>PANASONIC (P)</v>
+      </c>
+      <c r="D1278" t="str">
+        <v/>
+      </c>
+      <c r="E1278" t="str">
+        <v>Phase 3</v>
+      </c>
+      <c r="F1278" t="str">
+        <v/>
+      </c>
+      <c r="G1278">
+        <v>0.45</v>
+      </c>
+      <c r="H1278">
+        <v>1000</v>
+      </c>
+      <c r="I1278" t="str">
+        <v/>
+      </c>
+      <c r="J1278">
+        <v>1000</v>
+      </c>
+      <c r="K1278" t="str">
+        <v/>
+      </c>
+      <c r="L1278" t="str">
+        <v/>
+      </c>
+      <c r="M1278" t="str">
+        <v/>
+      </c>
+      <c r="N1278" t="str">
+        <v/>
+      </c>
+      <c r="O1278" t="str">
+        <v/>
+      </c>
+      <c r="P1278" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1277"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1278"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Accumulated updates: LAM 3PL, shared modules, workflow handlers
- LAM 3PL: roster updates, escalations, MPN switches, reorder/rfq-writer changes
- shared/: API client improvements, throttling, retry policy, daily counter
- shared/: email-workflow-poller, franchise-api, load-bulk-summary, vq-writer
- workflow-actions/: updates across all handlers (approval, broker-offers, excess,
  lam-kitting, rfq-loading, stockrfq, stockrfq-cq, tracking-loading, vq-loading)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -2489,7 +2489,7 @@
         <v>57.9390243902439</v>
       </c>
       <c r="H36">
-        <v>10</v>
+        <v>250</v>
       </c>
       <c r="I36" t="str">
         <v>28 weeks</v>
@@ -6796,7 +6796,7 @@
         <v>0.476829268292683</v>
       </c>
       <c r="H109">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="I109" t="str">
         <v>5 weeks</v>
@@ -7150,7 +7150,7 @@
         <v/>
       </c>
       <c r="H115">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I115" t="str">
         <v/>
@@ -7209,7 +7209,7 @@
         <v/>
       </c>
       <c r="H116">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I116" t="str">
         <v/>
@@ -7268,7 +7268,7 @@
         <v/>
       </c>
       <c r="H117">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I117" t="str">
         <v/>
@@ -7327,7 +7327,7 @@
         <v/>
       </c>
       <c r="H118">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I118" t="str">
         <v/>
@@ -11398,7 +11398,7 @@
         <v/>
       </c>
       <c r="H187">
-        <v>235</v>
+        <v>100</v>
       </c>
       <c r="I187" t="str">
         <v/>
@@ -11457,7 +11457,7 @@
         <v/>
       </c>
       <c r="H188">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="I188" t="str">
         <v/>
@@ -11516,7 +11516,7 @@
         <v/>
       </c>
       <c r="H189">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I189" t="str">
         <v/>
@@ -11575,7 +11575,7 @@
         <v/>
       </c>
       <c r="H190">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="I190" t="str">
         <v/>
@@ -13227,7 +13227,7 @@
         <v>0.43</v>
       </c>
       <c r="H218">
-        <v>5</v>
+        <v>750</v>
       </c>
       <c r="I218" t="str">
         <v>20 WEEKS</v>
@@ -16118,7 +16118,7 @@
         <v/>
       </c>
       <c r="H267">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I267" t="str">
         <v/>
@@ -17298,7 +17298,7 @@
         <v/>
       </c>
       <c r="H287">
-        <v>205</v>
+        <v>20</v>
       </c>
       <c r="I287" t="str">
         <v/>
@@ -29983,7 +29983,7 @@
         <v>104.67</v>
       </c>
       <c r="H502">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I502" t="str">
         <v>17 WEEKS</v>
@@ -46149,7 +46149,7 @@
         <v>12.34668780487805</v>
       </c>
       <c r="H776">
-        <v>2000</v>
+        <v>20</v>
       </c>
       <c r="I776" t="str">
         <v>21 Weeks</v>
@@ -47388,7 +47388,7 @@
         <v/>
       </c>
       <c r="H797">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I797" t="str">
         <v/>
@@ -69690,7 +69690,7 @@
         <v/>
       </c>
       <c r="H1175">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="I1175" t="str">
         <v>5 weeks</v>
@@ -69749,7 +69749,7 @@
         <v/>
       </c>
       <c r="H1176">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="I1176" t="str">
         <v>5 weeks</v>
@@ -69808,7 +69808,7 @@
         <v/>
       </c>
       <c r="H1177">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I1177" t="str">
         <v>5 weeks</v>
@@ -69867,7 +69867,7 @@
         <v/>
       </c>
       <c r="H1178">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I1178" t="str">
         <v>5 weeks</v>
@@ -69926,7 +69926,7 @@
         <v/>
       </c>
       <c r="H1179">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I1179" t="str">
         <v>5 weeks</v>
@@ -69985,7 +69985,7 @@
         <v/>
       </c>
       <c r="H1180">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I1180" t="str">
         <v>5 weeks</v>
@@ -70044,7 +70044,7 @@
         <v/>
       </c>
       <c r="H1181">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="I1181" t="str">
         <v/>
@@ -70103,7 +70103,7 @@
         <v/>
       </c>
       <c r="H1182">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="I1182" t="str">
         <v/>
@@ -71578,7 +71578,7 @@
         <v/>
       </c>
       <c r="H1207">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="I1207" t="str">
         <v/>
@@ -71619,7 +71619,7 @@
         <v/>
       </c>
       <c r="H1208">
-        <v>1</v>
+        <v>5000</v>
       </c>
       <c r="I1208" t="str">
         <v/>
@@ -71659,8 +71659,8 @@
       <c r="G1209" t="str">
         <v/>
       </c>
-      <c r="H1209" t="str">
-        <v/>
+      <c r="H1209">
+        <v>250</v>
       </c>
       <c r="I1209" t="str">
         <v/>
@@ -71700,8 +71700,8 @@
       <c r="G1210" t="str">
         <v/>
       </c>
-      <c r="H1210" t="str">
-        <v/>
+      <c r="H1210">
+        <v>250</v>
       </c>
       <c r="I1210" t="str">
         <v/>
@@ -71741,8 +71741,8 @@
       <c r="G1211" t="str">
         <v/>
       </c>
-      <c r="H1211" t="str">
-        <v/>
+      <c r="H1211">
+        <v>500</v>
       </c>
       <c r="I1211" t="str">
         <v/>
@@ -71783,7 +71783,7 @@
         <v/>
       </c>
       <c r="H1212">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1212" t="str">
         <v/>
@@ -71823,8 +71823,8 @@
       <c r="G1213" t="str">
         <v/>
       </c>
-      <c r="H1213" t="str">
-        <v/>
+      <c r="H1213">
+        <v>250</v>
       </c>
       <c r="I1213" t="str">
         <v/>
@@ -71865,7 +71865,7 @@
         <v/>
       </c>
       <c r="H1214">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1214" t="str">
         <v/>
@@ -71905,8 +71905,8 @@
       <c r="G1215" t="str">
         <v/>
       </c>
-      <c r="H1215" t="str">
-        <v/>
+      <c r="H1215">
+        <v>50</v>
       </c>
       <c r="I1215" t="str">
         <v/>
@@ -71988,7 +71988,7 @@
         <v/>
       </c>
       <c r="H1217">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1217" t="str">
         <v/>
@@ -72029,7 +72029,7 @@
         <v/>
       </c>
       <c r="H1218">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="I1218" t="str">
         <v/>
@@ -72070,7 +72070,7 @@
         <v/>
       </c>
       <c r="H1219">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1219" t="str">
         <v/>
@@ -72111,7 +72111,7 @@
         <v/>
       </c>
       <c r="H1220">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="I1220" t="str">
         <v/>
@@ -72152,7 +72152,7 @@
         <v/>
       </c>
       <c r="H1221">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="I1221" t="str">
         <v/>
@@ -72193,7 +72193,7 @@
         <v/>
       </c>
       <c r="H1222">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1222" t="str">
         <v/>
@@ -72234,7 +72234,7 @@
         <v/>
       </c>
       <c r="H1223">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="I1223" t="str">
         <v/>
@@ -72275,7 +72275,7 @@
         <v/>
       </c>
       <c r="H1224">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="I1224" t="str">
         <v/>
@@ -72316,7 +72316,7 @@
         <v/>
       </c>
       <c r="H1225">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1225" t="str">
         <v/>
@@ -72357,7 +72357,7 @@
         <v/>
       </c>
       <c r="H1226">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1226" t="str">
         <v/>
@@ -72398,7 +72398,7 @@
         <v/>
       </c>
       <c r="H1227">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1227" t="str">
         <v/>
@@ -72479,8 +72479,8 @@
       <c r="G1229" t="str">
         <v/>
       </c>
-      <c r="H1229" t="str">
-        <v/>
+      <c r="H1229">
+        <v>10</v>
       </c>
       <c r="I1229" t="str">
         <v/>
@@ -72521,7 +72521,7 @@
         <v/>
       </c>
       <c r="H1230">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="I1230" t="str">
         <v/>
@@ -72562,7 +72562,7 @@
         <v/>
       </c>
       <c r="H1231">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="I1231" t="str">
         <v/>
@@ -72603,7 +72603,7 @@
         <v/>
       </c>
       <c r="H1232">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1232" t="str">
         <v/>
@@ -72644,7 +72644,7 @@
         <v/>
       </c>
       <c r="H1233">
-        <v>1</v>
+        <v>4000</v>
       </c>
       <c r="I1233" t="str">
         <v/>
@@ -72685,7 +72685,7 @@
         <v/>
       </c>
       <c r="H1234">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I1234" t="str">
         <v/>
@@ -72726,7 +72726,7 @@
         <v/>
       </c>
       <c r="H1235">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="I1235" t="str">
         <v/>
@@ -72767,7 +72767,7 @@
         <v/>
       </c>
       <c r="H1236">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="I1236" t="str">
         <v/>
@@ -72808,7 +72808,7 @@
         <v/>
       </c>
       <c r="H1237">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="I1237" t="str">
         <v/>
@@ -72849,7 +72849,7 @@
         <v/>
       </c>
       <c r="H1238">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="I1238" t="str">
         <v/>
@@ -72890,7 +72890,7 @@
         <v/>
       </c>
       <c r="H1239">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="I1239" t="str">
         <v/>
@@ -72931,7 +72931,7 @@
         <v>6.853658536585367</v>
       </c>
       <c r="H1240">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="I1240" t="str">
         <v>5 weeks</v>
@@ -72972,7 +72972,7 @@
         <v/>
       </c>
       <c r="H1241">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I1241" t="str">
         <v/>
@@ -73013,7 +73013,7 @@
         <v/>
       </c>
       <c r="H1242">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I1242" t="str">
         <v/>
@@ -73054,7 +73054,7 @@
         <v/>
       </c>
       <c r="H1243">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1243" t="str">
         <v/>
@@ -73094,8 +73094,8 @@
       <c r="G1244" t="str">
         <v/>
       </c>
-      <c r="H1244" t="str">
-        <v/>
+      <c r="H1244">
+        <v>100</v>
       </c>
       <c r="I1244" t="str">
         <v/>
@@ -73136,7 +73136,7 @@
         <v/>
       </c>
       <c r="H1245">
-        <v>1</v>
+        <v>1500</v>
       </c>
       <c r="I1245" t="str">
         <v/>
@@ -73177,7 +73177,7 @@
         <v/>
       </c>
       <c r="H1246">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="I1246" t="str">
         <v/>
@@ -73300,7 +73300,7 @@
         <v/>
       </c>
       <c r="H1249">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I1249" t="str">
         <v/>

</xml_diff>

<commit_message>
Fix Phase 3 row-offset corruption and toFixed error
Root cause: Phase 3 onboarding on 2026-07-17 had CPC→MPN shifted
by one row. This corrupted data propagated through all subsequent
sourced files.

Fixes:
1. MPN now updates from fresh roster on each merge (otColumns)
2. Fixed toFixed() error when margin value is string not number
3. Reverted stale API clearing (was too aggressive)

Full run with fresh APIs now produces correct CPC→MPN associations.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S1254"/>
+  <dimension ref="A1:S1255"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -71581,16 +71581,19 @@
         <v>10000</v>
       </c>
       <c r="I1207" t="str">
-        <v/>
+        <v>20 weeks</v>
       </c>
       <c r="J1207" t="str">
         <v/>
+      </c>
+      <c r="P1207" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1207" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1207" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1207" t="str">
         <v>N/A</v>
@@ -71601,10 +71604,10 @@
         <v>615-068556-200</v>
       </c>
       <c r="B1208" t="str">
-        <v>CX480D5</v>
+        <v>ERJ-3RQF2R0V</v>
       </c>
       <c r="C1208" t="str">
-        <v>CRYDOM (P)</v>
+        <v>PANASONIC (P)</v>
       </c>
       <c r="D1208" t="str">
         <v/>
@@ -71613,7 +71616,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1208">
-        <v>31.31</v>
+        <v>0.11</v>
       </c>
       <c r="G1208" t="str">
         <v/>
@@ -71622,16 +71625,19 @@
         <v>5000</v>
       </c>
       <c r="I1208" t="str">
-        <v/>
+        <v>24 weeks</v>
       </c>
       <c r="J1208" t="str">
         <v/>
+      </c>
+      <c r="P1208" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1208" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1208" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1208" t="str">
         <v>N/A</v>
@@ -71663,16 +71669,19 @@
         <v>250</v>
       </c>
       <c r="I1209" t="str">
-        <v/>
+        <v>13 weeks</v>
       </c>
       <c r="J1209" t="str">
         <v/>
+      </c>
+      <c r="P1209" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1209" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1209" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1209" t="str">
         <v>N/A</v>
@@ -71704,16 +71713,19 @@
         <v>250</v>
       </c>
       <c r="I1210" t="str">
-        <v/>
+        <v>13 weeks</v>
       </c>
       <c r="J1210" t="str">
         <v/>
+      </c>
+      <c r="P1210" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1210" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1210" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1210" t="str">
         <v>N/A</v>
@@ -71745,16 +71757,19 @@
         <v>500</v>
       </c>
       <c r="I1211" t="str">
-        <v/>
+        <v>13 weeks</v>
       </c>
       <c r="J1211" t="str">
         <v/>
+      </c>
+      <c r="P1211" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1211" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1211" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1211" t="str">
         <v>N/A</v>
@@ -71765,10 +71780,10 @@
         <v>615-224835-010</v>
       </c>
       <c r="B1212" t="str">
-        <v>C3216X7R1V475K160AB</v>
+        <v>PATT0603E4991BGT1</v>
       </c>
       <c r="C1212" t="str">
-        <v>TDK (P)</v>
+        <v>VISHAY (P)</v>
       </c>
       <c r="D1212" t="str">
         <v/>
@@ -71777,7 +71792,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1212">
-        <v>0.63</v>
+        <v>0.89</v>
       </c>
       <c r="G1212" t="str">
         <v/>
@@ -71786,16 +71801,19 @@
         <v>1000</v>
       </c>
       <c r="I1212" t="str">
-        <v/>
+        <v>31 weeks</v>
       </c>
       <c r="J1212" t="str">
         <v/>
+      </c>
+      <c r="P1212" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1212" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1212" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1212" t="str">
         <v>N/A</v>
@@ -71827,16 +71845,19 @@
         <v>250</v>
       </c>
       <c r="I1213" t="str">
-        <v/>
+        <v>10 weeks</v>
       </c>
       <c r="J1213" t="str">
         <v/>
+      </c>
+      <c r="P1213" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1213" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1213" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1213" t="str">
         <v>N/A</v>
@@ -71868,16 +71889,19 @@
         <v>100</v>
       </c>
       <c r="I1214" t="str">
-        <v/>
+        <v>31 weeks</v>
       </c>
       <c r="J1214" t="str">
         <v/>
+      </c>
+      <c r="P1214" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1214" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1214" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1214" t="str">
         <v>N/A</v>
@@ -71909,16 +71933,19 @@
         <v>50</v>
       </c>
       <c r="I1215" t="str">
-        <v/>
+        <v>15 weeks</v>
       </c>
       <c r="J1215" t="str">
         <v/>
+      </c>
+      <c r="P1215" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1215" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1215" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1215" t="str">
         <v>N/A</v>
@@ -71959,7 +71986,7 @@
         <v>2026-07-17</v>
       </c>
       <c r="R1216" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1216" t="str">
         <v>N/A</v>
@@ -71970,10 +71997,10 @@
         <v>630-096581-001</v>
       </c>
       <c r="B1217" t="str">
-        <v>555-2401F</v>
+        <v>LT1013DS8#PBF</v>
       </c>
       <c r="C1217" t="str">
-        <v>DIALIGHT (P)</v>
+        <v>ANALOG DEVICES INC. (P)</v>
       </c>
       <c r="D1217" t="str">
         <v/>
@@ -71982,7 +72009,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1217">
-        <v>1.59</v>
+        <v>6.98</v>
       </c>
       <c r="G1217" t="str">
         <v/>
@@ -71991,16 +72018,19 @@
         <v>100</v>
       </c>
       <c r="I1217" t="str">
-        <v/>
+        <v>21 weeks</v>
       </c>
       <c r="J1217" t="str">
         <v/>
+      </c>
+      <c r="P1217" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1217" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1217" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1217" t="str">
         <v>N/A</v>
@@ -72032,16 +72062,19 @@
         <v>200</v>
       </c>
       <c r="I1218" t="str">
-        <v/>
+        <v>27 weeks</v>
       </c>
       <c r="J1218" t="str">
         <v/>
+      </c>
+      <c r="P1218" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1218" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1218" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1218" t="str">
         <v>N/A</v>
@@ -72052,10 +72085,10 @@
         <v>630-212275-001</v>
       </c>
       <c r="B1219" t="str">
-        <v>DP83630SQ/NOPB</v>
+        <v>L6491</v>
       </c>
       <c r="C1219" t="str">
-        <v>TEXAS INSTRUMENTS (P)</v>
+        <v>STMICROELECTRONICS (P)</v>
       </c>
       <c r="D1219" t="str">
         <v/>
@@ -72064,7 +72097,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1219">
-        <v>12.64</v>
+        <v>2.85</v>
       </c>
       <c r="G1219" t="str">
         <v/>
@@ -72073,16 +72106,19 @@
         <v>100</v>
       </c>
       <c r="I1219" t="str">
-        <v/>
+        <v>18 weeks</v>
       </c>
       <c r="J1219" t="str">
         <v/>
+      </c>
+      <c r="P1219" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1219" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1219" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1219" t="str">
         <v>N/A</v>
@@ -72114,16 +72150,19 @@
         <v>150</v>
       </c>
       <c r="I1220" t="str">
-        <v/>
+        <v>34 weeks</v>
       </c>
       <c r="J1220" t="str">
         <v/>
+      </c>
+      <c r="P1220" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1220" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1220" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1220" t="str">
         <v>N/A</v>
@@ -72155,16 +72194,19 @@
         <v>30</v>
       </c>
       <c r="I1221" t="str">
-        <v/>
+        <v>18 weeks</v>
       </c>
       <c r="J1221" t="str">
         <v/>
+      </c>
+      <c r="P1221" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1221" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1221" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1221" t="str">
         <v>N/A</v>
@@ -72196,16 +72238,19 @@
         <v>100</v>
       </c>
       <c r="I1222" t="str">
-        <v/>
+        <v>12 weeks</v>
       </c>
       <c r="J1222" t="str">
         <v/>
+      </c>
+      <c r="P1222" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1222" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1222" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1222" t="str">
         <v>N/A</v>
@@ -72237,16 +72282,19 @@
         <v>150</v>
       </c>
       <c r="I1223" t="str">
-        <v/>
+        <v>12 weeks</v>
       </c>
       <c r="J1223" t="str">
         <v/>
+      </c>
+      <c r="P1223" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1223" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1223" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1223" t="str">
         <v>N/A</v>
@@ -72257,7 +72305,7 @@
         <v>630-265677-001</v>
       </c>
       <c r="B1224" t="str">
-        <v>TPS26620DRCT</v>
+        <v>LM2941SX/NOPB</v>
       </c>
       <c r="C1224" t="str">
         <v>TEXAS INSTRUMENTS (P)</v>
@@ -72269,7 +72317,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1224">
-        <v>2.61</v>
+        <v>1.49</v>
       </c>
       <c r="G1224" t="str">
         <v/>
@@ -72278,16 +72326,19 @@
         <v>500</v>
       </c>
       <c r="I1224" t="str">
-        <v/>
+        <v>12 weeks</v>
       </c>
       <c r="J1224" t="str">
         <v/>
+      </c>
+      <c r="P1224" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1224" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1224" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1224" t="str">
         <v>N/A</v>
@@ -72298,10 +72349,10 @@
         <v>630-272519-001</v>
       </c>
       <c r="B1225" t="str">
-        <v>ECEA1VKS470</v>
+        <v>OPA2192IDGKT</v>
       </c>
       <c r="C1225" t="str">
-        <v>Panasonic</v>
+        <v>TEXAS INSTRUMENTS (P)</v>
       </c>
       <c r="D1225" t="str">
         <v/>
@@ -72310,7 +72361,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1225">
-        <v>0.45</v>
+        <v>5.34</v>
       </c>
       <c r="G1225" t="str">
         <v/>
@@ -72319,16 +72370,19 @@
         <v>250</v>
       </c>
       <c r="I1225" t="str">
-        <v/>
+        <v>14 weeks</v>
       </c>
       <c r="J1225" t="str">
         <v/>
+      </c>
+      <c r="P1225" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1225" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1225" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1225" t="str">
         <v>N/A</v>
@@ -72339,10 +72393,10 @@
         <v>630-311553-001</v>
       </c>
       <c r="B1226" t="str">
-        <v>40.1151</v>
+        <v>DP83630SQ/NOPB</v>
       </c>
       <c r="C1226" t="str">
-        <v>SCHURTER (P)</v>
+        <v>TEXAS INSTRUMENTS (P)</v>
       </c>
       <c r="D1226" t="str">
         <v/>
@@ -72351,7 +72405,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1226">
-        <v>9.32</v>
+        <v>12.64</v>
       </c>
       <c r="G1226" t="str">
         <v/>
@@ -72360,16 +72414,19 @@
         <v>100</v>
       </c>
       <c r="I1226" t="str">
-        <v/>
+        <v>6 weeks</v>
       </c>
       <c r="J1226" t="str">
         <v/>
+      </c>
+      <c r="P1226" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1226" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1226" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1226" t="str">
         <v>N/A</v>
@@ -72380,7 +72437,7 @@
         <v>630-341490-001</v>
       </c>
       <c r="B1227" t="str">
-        <v>OPA2192IDGKT</v>
+        <v>TPS26620DRCT</v>
       </c>
       <c r="C1227" t="str">
         <v>TEXAS INSTRUMENTS (P)</v>
@@ -72392,7 +72449,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1227">
-        <v>5.34</v>
+        <v>2.61</v>
       </c>
       <c r="G1227" t="str">
         <v/>
@@ -72401,16 +72458,19 @@
         <v>250</v>
       </c>
       <c r="I1227" t="str">
-        <v/>
+        <v>6 weeks</v>
       </c>
       <c r="J1227" t="str">
         <v/>
+      </c>
+      <c r="P1227" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1227" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1227" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1227" t="str">
         <v>N/A</v>
@@ -72439,19 +72499,22 @@
         <v/>
       </c>
       <c r="H1228">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="I1228" t="str">
-        <v/>
+        <v>42 weeks</v>
       </c>
       <c r="J1228" t="str">
         <v/>
+      </c>
+      <c r="P1228" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1228" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1228" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1228" t="str">
         <v>N/A</v>
@@ -72483,16 +72546,19 @@
         <v>10</v>
       </c>
       <c r="I1229" t="str">
-        <v/>
+        <v>9 weeks</v>
       </c>
       <c r="J1229" t="str">
         <v/>
+      </c>
+      <c r="P1229" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1229" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1229" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1229" t="str">
         <v>N/A</v>
@@ -72503,10 +72569,10 @@
         <v>639-B70524-101</v>
       </c>
       <c r="B1230" t="str">
-        <v>PATT0603E4991BGT1</v>
+        <v>SRR1208-101KL</v>
       </c>
       <c r="C1230" t="str">
-        <v>Vishay</v>
+        <v>BOURNS (P)</v>
       </c>
       <c r="D1230" t="str">
         <v/>
@@ -72515,7 +72581,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1230">
-        <v>0.89</v>
+        <v>1.29</v>
       </c>
       <c r="G1230" t="str">
         <v/>
@@ -72524,16 +72590,19 @@
         <v>400</v>
       </c>
       <c r="I1230" t="str">
-        <v/>
+        <v>23 weeks</v>
       </c>
       <c r="J1230" t="str">
         <v/>
+      </c>
+      <c r="P1230" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1230" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1230" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1230" t="str">
         <v>N/A</v>
@@ -72544,10 +72613,10 @@
         <v>644-338613-001</v>
       </c>
       <c r="B1231" t="str">
-        <v>LT1013DS8#PBF</v>
+        <v>CX480D5</v>
       </c>
       <c r="C1231" t="str">
-        <v>ANALOG DEVICES INC. (P)</v>
+        <v>CRYDOM (P)</v>
       </c>
       <c r="D1231" t="str">
         <v/>
@@ -72556,25 +72625,28 @@
         <v>Phase 3</v>
       </c>
       <c r="F1231">
-        <v>6.98</v>
+        <v>31.31</v>
       </c>
       <c r="G1231" t="str">
         <v/>
       </c>
       <c r="H1231">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="I1231" t="str">
-        <v/>
+        <v>10 weeks</v>
       </c>
       <c r="J1231" t="str">
         <v/>
+      </c>
+      <c r="P1231" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1231" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1231" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1231" t="str">
         <v>N/A</v>
@@ -72585,10 +72657,10 @@
         <v>648-130628-001</v>
       </c>
       <c r="B1232" t="str">
-        <v>LM2941SX/NOPB</v>
+        <v>EMVH500ADA101MJA0G</v>
       </c>
       <c r="C1232" t="str">
-        <v>TEXAS INSTRUMENTS (P)</v>
+        <v>NIPPON CHEMI-CON CORPORATION (P)</v>
       </c>
       <c r="D1232" t="str">
         <v/>
@@ -72597,7 +72669,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1232">
-        <v>1.49</v>
+        <v>0.39</v>
       </c>
       <c r="G1232" t="str">
         <v/>
@@ -72611,11 +72683,14 @@
       <c r="J1232" t="str">
         <v/>
       </c>
+      <c r="P1232" t="str">
+        <v>2026-07-30</v>
+      </c>
       <c r="Q1232" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1232" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1232" t="str">
         <v>N/A</v>
@@ -72626,10 +72701,10 @@
         <v>648-162696-004</v>
       </c>
       <c r="B1233" t="str">
-        <v>SRR1208-101KL</v>
+        <v>C1608X5R1V474K080AB</v>
       </c>
       <c r="C1233" t="str">
-        <v>BOURNS (P)</v>
+        <v>TDK (P)</v>
       </c>
       <c r="D1233" t="str">
         <v/>
@@ -72638,7 +72713,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1233">
-        <v>1.29</v>
+        <v>0.15</v>
       </c>
       <c r="G1233" t="str">
         <v/>
@@ -72647,16 +72722,19 @@
         <v>4000</v>
       </c>
       <c r="I1233" t="str">
-        <v/>
+        <v>24 weeks</v>
       </c>
       <c r="J1233" t="str">
         <v/>
+      </c>
+      <c r="P1233" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1233" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1233" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1233" t="str">
         <v>N/A</v>
@@ -72688,16 +72766,19 @@
         <v>10</v>
       </c>
       <c r="I1234" t="str">
-        <v/>
+        <v>8 weeks</v>
       </c>
       <c r="J1234" t="str">
         <v/>
+      </c>
+      <c r="P1234" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1234" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1234" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1234" t="str">
         <v>N/A</v>
@@ -72729,16 +72810,19 @@
         <v>200</v>
       </c>
       <c r="I1235" t="str">
-        <v/>
+        <v>28 weeks</v>
       </c>
       <c r="J1235" t="str">
         <v/>
+      </c>
+      <c r="P1235" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1235" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1235" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1235" t="str">
         <v>N/A</v>
@@ -72749,10 +72833,10 @@
         <v>648-314833-001</v>
       </c>
       <c r="B1236" t="str">
-        <v>164A16579X</v>
+        <v>C3216X7R1V475K160AB</v>
       </c>
       <c r="C1236" t="str">
-        <v>CONEC Elektronische Bauelemente GmbH</v>
+        <v>TDK (P)</v>
       </c>
       <c r="D1236" t="str">
         <v/>
@@ -72761,7 +72845,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1236">
-        <v>9.8</v>
+        <v>0.63</v>
       </c>
       <c r="G1236" t="str">
         <v/>
@@ -72770,16 +72854,19 @@
         <v>2000</v>
       </c>
       <c r="I1236" t="str">
-        <v/>
+        <v>25 weeks</v>
       </c>
       <c r="J1236" t="str">
         <v/>
+      </c>
+      <c r="P1236" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1236" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1236" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1236" t="str">
         <v>N/A</v>
@@ -72811,16 +72898,19 @@
         <v>260</v>
       </c>
       <c r="I1237" t="str">
-        <v/>
+        <v>48 weeks</v>
       </c>
       <c r="J1237" t="str">
         <v/>
+      </c>
+      <c r="P1237" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1237" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1237" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1237" t="str">
         <v>N/A</v>
@@ -72852,16 +72942,19 @@
         <v>40</v>
       </c>
       <c r="I1238" t="str">
-        <v/>
+        <v>20 weeks</v>
       </c>
       <c r="J1238" t="str">
         <v/>
+      </c>
+      <c r="P1238" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1238" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1238" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1238" t="str">
         <v>N/A</v>
@@ -72872,10 +72965,10 @@
         <v>662-060106-012</v>
       </c>
       <c r="B1239" t="str">
-        <v>EMVH500ADA101MJA0G</v>
+        <v>555-2401F</v>
       </c>
       <c r="C1239" t="str">
-        <v>Nippon Chemi-Con Corporation</v>
+        <v>DIALIGHT (P)</v>
       </c>
       <c r="D1239" t="str">
         <v/>
@@ -72884,7 +72977,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1239">
-        <v>0.39</v>
+        <v>1.59</v>
       </c>
       <c r="G1239" t="str">
         <v/>
@@ -72893,16 +72986,19 @@
         <v>500</v>
       </c>
       <c r="I1239" t="str">
-        <v/>
+        <v>22 weeks</v>
       </c>
       <c r="J1239" t="str">
         <v/>
+      </c>
+      <c r="P1239" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1239" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1239" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1239" t="str">
         <v>N/A</v>
@@ -72913,10 +73009,10 @@
         <v>668-096777-009</v>
       </c>
       <c r="B1240" t="str">
-        <v>K85X-ED-9P-CBR</v>
+        <v>DLS 1XP4AA35X</v>
       </c>
       <c r="C1240" t="str">
-        <v>KYCON, INC</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH</v>
       </c>
       <c r="D1240" t="str">
         <v>CONN,DSUB,9P,M,STR,BRD LCK,ROHS</v>
@@ -72934,16 +73030,19 @@
         <v>500</v>
       </c>
       <c r="I1240" t="str">
-        <v>5 weeks</v>
+        <v>14 weeks</v>
       </c>
       <c r="J1240" t="str">
         <v/>
+      </c>
+      <c r="P1240" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1240" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1240" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1240" t="str">
         <v>N/A</v>
@@ -72954,10 +73053,10 @@
         <v>668-132368-015</v>
       </c>
       <c r="B1241" t="str">
-        <v>ERJ-3RQF2R0V</v>
+        <v>164A16579X</v>
       </c>
       <c r="C1241" t="str">
-        <v>Panasonic</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH (P)</v>
       </c>
       <c r="D1241" t="str">
         <v/>
@@ -72966,7 +73065,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1241">
-        <v>0.11</v>
+        <v>9.8</v>
       </c>
       <c r="G1241" t="str">
         <v/>
@@ -72975,16 +73074,19 @@
         <v>50</v>
       </c>
       <c r="I1241" t="str">
-        <v/>
+        <v>15 weeks</v>
       </c>
       <c r="J1241" t="str">
         <v/>
+      </c>
+      <c r="P1241" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1241" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1241" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1241" t="str">
         <v>N/A</v>
@@ -72995,10 +73097,10 @@
         <v>668-C03283-001</v>
       </c>
       <c r="B1242" t="str">
-        <v>L6491</v>
+        <v>302W2CPXX72E40X</v>
       </c>
       <c r="C1242" t="str">
-        <v>STMICROELECTRONICS (P)</v>
+        <v>CONEC ELEKTRONISCHE BAUELEMENTE GMBH</v>
       </c>
       <c r="D1242" t="str">
         <v/>
@@ -73007,25 +73109,28 @@
         <v>Phase 3</v>
       </c>
       <c r="F1242">
-        <v>2.85</v>
+        <v>10.24</v>
       </c>
       <c r="G1242" t="str">
         <v/>
       </c>
       <c r="H1242">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="I1242" t="str">
-        <v/>
+        <v>14 weeks</v>
       </c>
       <c r="J1242" t="str">
         <v/>
+      </c>
+      <c r="P1242" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1242" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1242" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1242" t="str">
         <v>N/A</v>
@@ -73036,10 +73141,10 @@
         <v>671-084849-001</v>
       </c>
       <c r="B1243" t="str">
-        <v>C1608X5R1V474K080AB</v>
+        <v>40.1151</v>
       </c>
       <c r="C1243" t="str">
-        <v>TDK (P)</v>
+        <v>SCHURTER (P)</v>
       </c>
       <c r="D1243" t="str">
         <v/>
@@ -73048,7 +73153,7 @@
         <v>Phase 3</v>
       </c>
       <c r="F1243">
-        <v>0.15</v>
+        <v>9.32</v>
       </c>
       <c r="G1243" t="str">
         <v/>
@@ -73057,16 +73162,19 @@
         <v>100</v>
       </c>
       <c r="I1243" t="str">
-        <v/>
+        <v>10 weeks</v>
       </c>
       <c r="J1243" t="str">
         <v/>
+      </c>
+      <c r="P1243" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1243" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1243" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1243" t="str">
         <v>N/A</v>
@@ -73098,16 +73206,19 @@
         <v>100</v>
       </c>
       <c r="I1244" t="str">
-        <v/>
+        <v>20 weeks</v>
       </c>
       <c r="J1244" t="str">
         <v/>
+      </c>
+      <c r="P1244" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1244" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1244" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1244" t="str">
         <v>N/A</v>
@@ -73139,16 +73250,19 @@
         <v>1500</v>
       </c>
       <c r="I1245" t="str">
-        <v/>
+        <v>13 weeks</v>
       </c>
       <c r="J1245" t="str">
         <v/>
+      </c>
+      <c r="P1245" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1245" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1245" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1245" t="str">
         <v>N/A</v>
@@ -73180,16 +73294,19 @@
         <v>1000</v>
       </c>
       <c r="I1246" t="str">
-        <v/>
+        <v>13 weeks</v>
       </c>
       <c r="J1246" t="str">
         <v/>
+      </c>
+      <c r="P1246" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1246" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1246" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1246" t="str">
         <v>N/A</v>
@@ -73218,7 +73335,7 @@
         <v>42.4390243902439</v>
       </c>
       <c r="H1247">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I1247" t="str">
         <v>10 weeks</v>
@@ -73226,11 +73343,14 @@
       <c r="J1247" t="str">
         <v/>
       </c>
+      <c r="P1247" t="str">
+        <v>2026-07-30</v>
+      </c>
       <c r="Q1247" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1247" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1247" t="str">
         <v>N/A</v>
@@ -73262,16 +73382,19 @@
         <v>140</v>
       </c>
       <c r="I1248" t="str">
-        <v/>
+        <v>16 weeks</v>
       </c>
       <c r="J1248">
         <v>140</v>
       </c>
+      <c r="P1248" t="str">
+        <v>2026-07-30</v>
+      </c>
       <c r="Q1248" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1248" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1248" t="str">
         <v>N/A</v>
@@ -73282,10 +73405,10 @@
         <v>785-088248-001</v>
       </c>
       <c r="B1249" t="str">
-        <v>302W2CPXX72E40X</v>
+        <v>ORDER TO SPECIFICATION</v>
       </c>
       <c r="C1249" t="str">
-        <v>CONEC Elektronische Bauelemente GmbH</v>
+        <v>ORDER TO SPECIFICATION (P)</v>
       </c>
       <c r="D1249" t="str">
         <v/>
@@ -73294,25 +73417,28 @@
         <v>Phase 3</v>
       </c>
       <c r="F1249">
-        <v>10.24</v>
+        <v>3.1</v>
       </c>
       <c r="G1249" t="str">
         <v/>
       </c>
       <c r="H1249">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I1249" t="str">
-        <v/>
+        <v>3 weeks</v>
       </c>
       <c r="J1249" t="str">
         <v/>
+      </c>
+      <c r="P1249" t="str">
+        <v>2026-07-30</v>
       </c>
       <c r="Q1249" t="str">
         <v>2026-07-17</v>
       </c>
       <c r="R1249" t="str">
-        <v>Email: FW: PO approval for PHASE 3</v>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1249" t="str">
         <v>N/A</v>
@@ -73371,7 +73497,7 @@
         <v/>
       </c>
       <c r="R1250" t="str">
-        <v/>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1250" t="str">
         <v/>
@@ -73430,7 +73556,7 @@
         <v/>
       </c>
       <c r="R1251" t="str">
-        <v/>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1251" t="str">
         <v/>
@@ -73489,7 +73615,7 @@
         <v/>
       </c>
       <c r="R1252" t="str">
-        <v/>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1252" t="str">
         <v/>
@@ -73548,7 +73674,7 @@
         <v/>
       </c>
       <c r="R1253" t="str">
-        <v/>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1253" t="str">
         <v/>
@@ -73607,15 +73733,74 @@
         <v/>
       </c>
       <c r="R1254" t="str">
-        <v/>
+        <v>source-files/2026-07-14_Phase3_PO_Approval.csv</v>
       </c>
       <c r="S1254" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="str">
+        <v>29-178970-00</v>
+      </c>
+      <c r="B1255" t="str">
+        <v>ECEA1VKS470</v>
+      </c>
+      <c r="C1255" t="str">
+        <v>Panasonic</v>
+      </c>
+      <c r="D1255" t="str">
+        <v/>
+      </c>
+      <c r="E1255">
+        <v>1000</v>
+      </c>
+      <c r="F1255">
+        <v>0.45</v>
+      </c>
+      <c r="G1255">
+        <v>0</v>
+      </c>
+      <c r="H1255">
+        <v>1000</v>
+      </c>
+      <c r="I1255" t="str">
+        <v>52 weeks</v>
+      </c>
+      <c r="J1255">
+        <v>0</v>
+      </c>
+      <c r="K1255" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1255" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1255" t="str">
+        <v/>
+      </c>
+      <c r="N1255" t="str">
+        <v/>
+      </c>
+      <c r="O1255" t="str">
+        <v/>
+      </c>
+      <c r="P1255" t="str">
+        <v>2026-07-30</v>
+      </c>
+      <c r="Q1255" t="str">
+        <v/>
+      </c>
+      <c r="R1255" t="str">
+        <v/>
+      </c>
+      <c r="S1255" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S1254"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S1255"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update LAM Master Roster + last-inventory-date sidecar (weekly cron state)
Routine data refresh from lam-kitting-runner.js cron activity — roster
edits + last-inventory-date tracking (per POV staleness prevention,
lam-3pl.md).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
+++ b/Trading Analysis/LAM 3PL/LAM_Master_Roster.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S1255"/>
+  <dimension ref="A1:S1264"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -73798,9 +73798,540 @@
         <v/>
       </c>
     </row>
+    <row r="1256">
+      <c r="A1256" t="str">
+        <v>645-A30352-001</v>
+      </c>
+      <c r="B1256" t="str">
+        <v>HTS 91-01-HB-C F-0-735</v>
+      </c>
+      <c r="C1256" t="str">
+        <v>BEHLKE</v>
+      </c>
+      <c r="D1256" t="str">
+        <v/>
+      </c>
+      <c r="E1256">
+        <v>5</v>
+      </c>
+      <c r="F1256">
+        <v>0</v>
+      </c>
+      <c r="G1256">
+        <v>0</v>
+      </c>
+      <c r="H1256">
+        <v>1</v>
+      </c>
+      <c r="I1256" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="J1256">
+        <v>0</v>
+      </c>
+      <c r="K1256" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1256" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1256" t="str">
+        <v/>
+      </c>
+      <c r="N1256" t="str">
+        <v/>
+      </c>
+      <c r="O1256" t="str">
+        <v/>
+      </c>
+      <c r="P1256" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1256" t="str">
+        <v/>
+      </c>
+      <c r="R1256" t="str">
+        <v/>
+      </c>
+      <c r="S1256" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="str">
+        <v>669-B78543-004</v>
+      </c>
+      <c r="B1257" t="str">
+        <v>10-737585-178</v>
+      </c>
+      <c r="C1257" t="str">
+        <v>Amphenol</v>
+      </c>
+      <c r="D1257" t="str">
+        <v/>
+      </c>
+      <c r="E1257">
+        <v>100</v>
+      </c>
+      <c r="F1257">
+        <v>5.07</v>
+      </c>
+      <c r="G1257">
+        <v>0</v>
+      </c>
+      <c r="H1257">
+        <v>100</v>
+      </c>
+      <c r="I1257" t="str">
+        <v>16 WEEKS</v>
+      </c>
+      <c r="J1257">
+        <v>0</v>
+      </c>
+      <c r="K1257" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1257" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1257" t="str">
+        <v/>
+      </c>
+      <c r="N1257" t="str">
+        <v/>
+      </c>
+      <c r="O1257" t="str">
+        <v/>
+      </c>
+      <c r="P1257" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1257" t="str">
+        <v/>
+      </c>
+      <c r="R1257" t="str">
+        <v/>
+      </c>
+      <c r="S1257" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="str">
+        <v>668-C32577-001</v>
+      </c>
+      <c r="B1258" t="str">
+        <v>2484639-1</v>
+      </c>
+      <c r="C1258" t="str">
+        <v>TE Connectivity</v>
+      </c>
+      <c r="D1258" t="str">
+        <v/>
+      </c>
+      <c r="E1258">
+        <v>100</v>
+      </c>
+      <c r="F1258">
+        <v>6.96</v>
+      </c>
+      <c r="G1258">
+        <v>0</v>
+      </c>
+      <c r="H1258">
+        <v>100</v>
+      </c>
+      <c r="I1258" t="str">
+        <v>15 WEEKS</v>
+      </c>
+      <c r="J1258">
+        <v>0</v>
+      </c>
+      <c r="K1258" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1258" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1258" t="str">
+        <v/>
+      </c>
+      <c r="N1258" t="str">
+        <v/>
+      </c>
+      <c r="O1258" t="str">
+        <v/>
+      </c>
+      <c r="P1258" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1258" t="str">
+        <v/>
+      </c>
+      <c r="R1258" t="str">
+        <v/>
+      </c>
+      <c r="S1258" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="str">
+        <v>648-162121-031</v>
+      </c>
+      <c r="B1259" t="str">
+        <v>C0603C271J5RACTU</v>
+      </c>
+      <c r="C1259" t="str">
+        <v>Kemet</v>
+      </c>
+      <c r="D1259" t="str">
+        <v/>
+      </c>
+      <c r="E1259">
+        <v>4000</v>
+      </c>
+      <c r="F1259">
+        <v>0.25</v>
+      </c>
+      <c r="G1259">
+        <v>0</v>
+      </c>
+      <c r="H1259">
+        <v>4000</v>
+      </c>
+      <c r="I1259" t="str">
+        <v>29 WEEKS</v>
+      </c>
+      <c r="J1259">
+        <v>0</v>
+      </c>
+      <c r="K1259" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1259" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1259" t="str">
+        <v/>
+      </c>
+      <c r="N1259" t="str">
+        <v/>
+      </c>
+      <c r="O1259" t="str">
+        <v/>
+      </c>
+      <c r="P1259" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1259" t="str">
+        <v/>
+      </c>
+      <c r="R1259" t="str">
+        <v/>
+      </c>
+      <c r="S1259" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="str">
+        <v>639-066560-124</v>
+      </c>
+      <c r="B1260" t="str">
+        <v>MSS1278-124KLD</v>
+      </c>
+      <c r="C1260" t="str">
+        <v>Coilcraft</v>
+      </c>
+      <c r="D1260" t="str">
+        <v/>
+      </c>
+      <c r="E1260">
+        <v>500</v>
+      </c>
+      <c r="F1260">
+        <v>2.58</v>
+      </c>
+      <c r="G1260">
+        <v>0</v>
+      </c>
+      <c r="H1260">
+        <v>500</v>
+      </c>
+      <c r="I1260" t="str">
+        <v>16 WEEKS</v>
+      </c>
+      <c r="J1260">
+        <v>0</v>
+      </c>
+      <c r="K1260" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1260" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1260" t="str">
+        <v/>
+      </c>
+      <c r="N1260" t="str">
+        <v/>
+      </c>
+      <c r="O1260" t="str">
+        <v/>
+      </c>
+      <c r="P1260" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1260" t="str">
+        <v/>
+      </c>
+      <c r="R1260" t="str">
+        <v/>
+      </c>
+      <c r="S1260" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="str">
+        <v>630-248784-001</v>
+      </c>
+      <c r="B1261" t="str">
+        <v>LTC2348CLX-16#PBF</v>
+      </c>
+      <c r="C1261" t="str">
+        <v>Analog Devices Inc</v>
+      </c>
+      <c r="D1261" t="str">
+        <v/>
+      </c>
+      <c r="E1261">
+        <v>40</v>
+      </c>
+      <c r="F1261">
+        <v>42.75</v>
+      </c>
+      <c r="G1261">
+        <v>0</v>
+      </c>
+      <c r="H1261">
+        <v>250</v>
+      </c>
+      <c r="I1261" t="str">
+        <v>14 WEEKS</v>
+      </c>
+      <c r="J1261">
+        <v>0</v>
+      </c>
+      <c r="K1261" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1261" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1261" t="str">
+        <v/>
+      </c>
+      <c r="N1261" t="str">
+        <v/>
+      </c>
+      <c r="O1261" t="str">
+        <v/>
+      </c>
+      <c r="P1261" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1261" t="str">
+        <v/>
+      </c>
+      <c r="R1261" t="str">
+        <v/>
+      </c>
+      <c r="S1261" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="str">
+        <v>630-129625-001</v>
+      </c>
+      <c r="B1262" t="str">
+        <v>TPS7A4700RGWT</v>
+      </c>
+      <c r="C1262" t="str">
+        <v>Texas Instruments</v>
+      </c>
+      <c r="D1262" t="str">
+        <v/>
+      </c>
+      <c r="E1262">
+        <v>250</v>
+      </c>
+      <c r="F1262">
+        <v>5.63</v>
+      </c>
+      <c r="G1262">
+        <v>0</v>
+      </c>
+      <c r="H1262">
+        <v>250</v>
+      </c>
+      <c r="I1262" t="str">
+        <v>16 WEEKS</v>
+      </c>
+      <c r="J1262">
+        <v>0</v>
+      </c>
+      <c r="K1262" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1262" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1262" t="str">
+        <v/>
+      </c>
+      <c r="N1262" t="str">
+        <v/>
+      </c>
+      <c r="O1262" t="str">
+        <v/>
+      </c>
+      <c r="P1262" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1262" t="str">
+        <v/>
+      </c>
+      <c r="R1262" t="str">
+        <v/>
+      </c>
+      <c r="S1262" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="str">
+        <v>615-900962-002</v>
+      </c>
+      <c r="B1263" t="str">
+        <v>HVCB2512FTD499K</v>
+      </c>
+      <c r="C1263" t="str">
+        <v>Stackpole Electronics Inc</v>
+      </c>
+      <c r="D1263" t="str">
+        <v/>
+      </c>
+      <c r="E1263">
+        <v>2000</v>
+      </c>
+      <c r="F1263">
+        <v>5.28</v>
+      </c>
+      <c r="G1263">
+        <v>0</v>
+      </c>
+      <c r="H1263">
+        <v>2000</v>
+      </c>
+      <c r="I1263" t="str">
+        <v>13 WEEKS</v>
+      </c>
+      <c r="J1263">
+        <v>0</v>
+      </c>
+      <c r="K1263" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1263" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1263" t="str">
+        <v/>
+      </c>
+      <c r="N1263" t="str">
+        <v/>
+      </c>
+      <c r="O1263" t="str">
+        <v/>
+      </c>
+      <c r="P1263" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1263" t="str">
+        <v/>
+      </c>
+      <c r="R1263" t="str">
+        <v/>
+      </c>
+      <c r="S1263" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="str">
+        <v>615-259564-004</v>
+      </c>
+      <c r="B1264" t="str">
+        <v>CRCW12101K78FKTA</v>
+      </c>
+      <c r="C1264" t="str">
+        <v>Vishay</v>
+      </c>
+      <c r="D1264" t="str">
+        <v/>
+      </c>
+      <c r="E1264">
+        <v>100</v>
+      </c>
+      <c r="F1264">
+        <v>0.33</v>
+      </c>
+      <c r="G1264">
+        <v>0</v>
+      </c>
+      <c r="H1264">
+        <v>5000</v>
+      </c>
+      <c r="I1264" t="str">
+        <v>15 WEEKS</v>
+      </c>
+      <c r="J1264">
+        <v>0</v>
+      </c>
+      <c r="K1264" t="str">
+        <v>Jake Harris</v>
+      </c>
+      <c r="L1264" t="str">
+        <v>New Award</v>
+      </c>
+      <c r="M1264" t="str">
+        <v/>
+      </c>
+      <c r="N1264" t="str">
+        <v/>
+      </c>
+      <c r="O1264" t="str">
+        <v/>
+      </c>
+      <c r="P1264" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="Q1264" t="str">
+        <v/>
+      </c>
+      <c r="R1264" t="str">
+        <v/>
+      </c>
+      <c r="S1264" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S1255"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S1264"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>